<commit_message>
test: log team membership scope defect
</commit_message>
<xml_diff>
--- a/07_Testing Plan/02_test_phase_5_6/PHASE_0_6_AUDIT_TRACKER.xlsx
+++ b/07_Testing Plan/02_test_phase_5_6/PHASE_0_6_AUDIT_TRACKER.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R922f3f3df913426d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Guide" sheetId="2" r:id="Rb01e0be59bb04da8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Plan" sheetId="3" r:id="R95ba0b4d6f504c42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carryover P0-4" sheetId="4" r:id="R76f40ec889604bfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 5 Scenarios" sheetId="5" r:id="R1f7494e133224fd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 6 Scenarios" sheetId="6" r:id="R102fc1099d694eea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="7" r:id="Rafeabfdf80964f36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R1b214e27a60a44f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Guide" sheetId="2" r:id="R6171b57647fa4c8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Plan" sheetId="3" r:id="R876163687d2c46b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carryover P0-4" sheetId="4" r:id="Rac4787d30275477b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 5 Scenarios" sheetId="5" r:id="Rf7fbeff35e6c4085"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 6 Scenarios" sheetId="6" r:id="Rfbc672800b1345a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="7" r:id="R67134e609a4246ff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -187,7 +187,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="92">
+  <x:cellXfs count="93">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -402,6 +402,7 @@
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -657,14 +658,14 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="B5" s="77" t="n">
-        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$64,A5)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A5)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A5)</x:f>
+        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$65,A5)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A5)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A5)</x:f>
         <x:v>67</x:v>
       </x:c>
       <x:c r="D5" s="77" t="str">
         <x:v>Carryover P0-4</x:v>
       </x:c>
       <x:c r="E5" s="77" t="n">
-        <x:v>60</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -672,7 +673,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="B6" s="77" t="n">
-        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$64,A6)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A6)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A6)</x:f>
+        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$65,A6)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A6)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A6)</x:f>
         <x:v>33</x:v>
       </x:c>
       <x:c r="D6" s="77" t="str">
@@ -687,8 +688,8 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="B7" s="77" t="n">
-        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$64,A7)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A7)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A7)</x:f>
-        <x:v>23</x:v>
+        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$65,A7)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A7)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A7)</x:f>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D7" s="77" t="str">
         <x:v>Phase 6 scenarios</x:v>
@@ -702,7 +703,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B8" s="77" t="n">
-        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$64,A8)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A8)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A8)</x:f>
+        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$65,A8)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A8)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A8)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="D8" s="77" t="str">
@@ -710,7 +711,7 @@
       </x:c>
       <x:c r="E8" s="77" t="n">
         <x:f>SUM(E5:E7)-B10-B11</x:f>
-        <x:v>178</x:v>
+        <x:v>179</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -718,7 +719,7 @@
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="B9" s="77" t="n">
-        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$64,A9)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A9)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A9)</x:f>
+        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$65,A9)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A9)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A9)</x:f>
         <x:v>41</x:v>
       </x:c>
       <x:c r="D9" s="77"/>
@@ -729,7 +730,7 @@
         <x:v>Future Backlog</x:v>
       </x:c>
       <x:c r="B10" s="77" t="n">
-        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$64,A10)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A10)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A10)</x:f>
+        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$65,A10)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A10)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A10)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="D10" s="77" t="str">
@@ -737,7 +738,7 @@
       </x:c>
       <x:c r="E10" s="89" t="n">
         <x:f>IF(E8=0,0,(E8-B9)/E8)</x:f>
-        <x:v>0.7696629213483146</x:v>
+        <x:v>0.770949720670391</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -745,7 +746,7 @@
         <x:v>Not Required</x:v>
       </x:c>
       <x:c r="B11" s="77" t="n">
-        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$64,A11)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A11)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A11)</x:f>
+        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$65,A11)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A11)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A11)</x:f>
         <x:v>4</x:v>
       </x:c>
     </x:row>
@@ -1316,7 +1317,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>60 unresolved, blocked, deferred or Future Backlog rows carried from DEVINT_PHASE_0_4_AUDIT_TRACKER.xlsx.</x:v>
+        <x:v>61 unresolved, blocked, deferred or Future Backlog rows carried from DEVINT Phase 0-4 audit.</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -2665,22 +2666,22 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="M25" s="51" t="str">
-        <x:v>Owner defaults to Unassigned, not the signed-in user. Signed-in Hieu is absent from owner options.</x:v>
+        <x:v>Owner defaults to Unassigned. After Hieu was added to Pegasus, Settings &gt; Teams showed Anh and Hieu, but the US-1 Owner dropdown still showed only No Entry and Anh. Owner membership options did not refresh from current Team membership.</x:v>
       </x:c>
       <x:c r="N25" s="51" t="str">
-        <x:v>evidence/retest_2026-07-24/P1-CREATE-01-quick-create.png</x:v>
+        <x:v>../Codex_audit_06_tracker.md</x:v>
       </x:c>
       <x:c r="O25" s="51" t="str">
-        <x:v>Fix default/allowed owner behavior per approved rule.</x:v>
+        <x:v>Keep the approved default rule. Source every Owner selector from current Project/Team membership and invalidate stale membership options after a member is added or removed.</x:v>
       </x:c>
       <x:c r="P25" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q25" s="51" t="str">
-        <x:v>Fix Direction Approved</x:v>
-      </x:c>
-      <x:c r="R25" s="56" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Bug confirmed; membership sync required</x:v>
+      </x:c>
+      <x:c r="R25" s="56" t="n">
+        <x:v>46240</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -5135,6 +5136,67 @@
       </x:c>
       <x:c r="R64" s="57" t="str">
         <x:v>2026-08-05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" t="str">
+        <x:v>GAP-P3-TS-008</x:v>
+      </x:c>
+      <x:c r="B65" t="str">
+        <x:v>Phase 3</x:v>
+      </x:c>
+      <x:c r="C65" t="str">
+        <x:v>Team Status</x:v>
+      </x:c>
+      <x:c r="D65" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E65" t="str">
+        <x:v>Team membership scope consistency</x:v>
+      </x:c>
+      <x:c r="F65" t="str">
+        <x:v>Signed in to DevInt. Project TEST, Team Pegasus and Iteration IT-1 are available. Team membership can be checked in Settings &gt; Teams.</x:v>
+      </x:c>
+      <x:c r="G65" t="str">
+        <x:v>Team Pegasus; users Anh and Hieu; US-1 and a Task assigned to Hieu. Compare the state before and after adding Hieu to Pegasus.</x:v>
+      </x:c>
+      <x:c r="H65" t="str">
+        <x:v>1. Check Pegasus membership in Settings &gt; Teams.
+2. Open Team Status in the same Project/Team/Iteration scope and compare member groups.
+3. Add Hieu to Pegasus.
+4. Reload Team Status and verify Hieu appears once.
+5. Open US-1 and inspect the Owner dropdown.
+6. Reload and confirm all views use the same current membership.</x:v>
+      </x:c>
+      <x:c r="I65" t="str">
+        <x:v>Team Status member groups and all Owner selectors use the same current Team membership source. A non-member is not presented as a current Team member. After an active member is added, that person becomes available in Owner selectors without stale data.</x:v>
+      </x:c>
+      <x:c r="J65" t="str">
+        <x:v>Phase 3/01_Team_Status/SRS.md; Phase 1/03_Work_Item_Detail/SRS.md</x:v>
+      </x:c>
+      <x:c r="K65" t="str">
+        <x:v>New defect found 2026-08-06</x:v>
+      </x:c>
+      <x:c r="L65" t="str">
+        <x:v>Fail</x:v>
+      </x:c>
+      <x:c r="M65" t="str">
+        <x:v>Hieu appeared in Team Status before belonging to Pegasus. After Hieu was added, Settings &gt; Teams and Team Status both showed Anh and Hieu, but the US-1 Owner dropdown still showed only No Entry and Anh.</x:v>
+      </x:c>
+      <x:c r="N65" t="str">
+        <x:v>../Codex_audit_06_tracker.md</x:v>
+      </x:c>
+      <x:c r="O65" t="str">
+        <x:v>Use one current Team-membership source for Team Status and Owner selectors, and refresh/invalidate membership caches after add/remove. Existing Task-owner treatment when a member is removed remains Pending BA.</x:v>
+      </x:c>
+      <x:c r="P65" t="str">
+        <x:v>BA + Codex</x:v>
+      </x:c>
+      <x:c r="Q65" t="str">
+        <x:v>Bug confirmed; removal behavior pending</x:v>
+      </x:c>
+      <x:c r="R65" s="92" t="n">
+        <x:v>46240</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -15368,15 +15430,33 @@
       </x:c>
     </x:row>
     <x:row r="66">
-      <x:c r="A66" s="86"/>
-      <x:c r="B66" s="83"/>
-      <x:c r="C66" s="83"/>
-      <x:c r="D66" s="83"/>
-      <x:c r="E66" s="83"/>
-      <x:c r="F66" s="83"/>
-      <x:c r="G66" s="83"/>
-      <x:c r="H66" s="83"/>
-      <x:c r="I66" s="73"/>
+      <x:c r="A66" s="86" t="n">
+        <x:v>46240</x:v>
+      </x:c>
+      <x:c r="B66" s="83" t="str">
+        <x:v>GAP-P3-TS-008</x:v>
+      </x:c>
+      <x:c r="C66" s="83" t="str">
+        <x:v>rally-dev.qnsc.vn</x:v>
+      </x:c>
+      <x:c r="D66" s="83" t="str">
+        <x:v>QNSC / TEST / Pegasus</x:v>
+      </x:c>
+      <x:c r="E66" s="83" t="str">
+        <x:v>BA + Codex</x:v>
+      </x:c>
+      <x:c r="F66" s="83" t="str">
+        <x:v>Fail</x:v>
+      </x:c>
+      <x:c r="G66" s="83" t="str">
+        <x:v>../Codex_audit_06_tracker.md</x:v>
+      </x:c>
+      <x:c r="H66" s="83" t="str">
+        <x:v>GAP-P3-TS-008</x:v>
+      </x:c>
+      <x:c r="I66" s="73" t="str">
+        <x:v>Team Status and Work Item Owner selectors used inconsistent/stale Team membership. Removed-member Task treatment remains Pending BA.</x:v>
+      </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="86"/>

</xml_diff>